<commit_message>
Planilha por ano: top 10
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQAEiUYJHrFswFx8FRgado
</commit_message>
<xml_diff>
--- a/top_anuncios_subido_ao_vivo_por_ano.xlsx
+++ b/top_anuncios_subido_ao_vivo_por_ano.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -697,29 +697,29 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AD65 - Carrossel 4 - Palestrantes confirmados</t>
+          <t>AD01 - Vídeo Feed 1</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>imagem</t>
+          <t>vídeo</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>934.12</v>
+        <v>7980.04</v>
       </c>
       <c r="F6" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>17.62</v>
+        <v>137.59</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.02719343252950231</v>
+        <v>0.0297588506926629</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] [ALUNO] [V2] Venda LOTE 2 - MAI/24</t>
+          <t>[PRE-INSCRICOES] [CADASTROS] [AUTO] [Q] Pré-inscrições LOTE 1 - FEV/24</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -727,7 +727,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C9c4mUht5FS/</t>
+          <t>https://www.instagram.com/p/C3FkNeQNkoM/</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AL01 - Vídeo SAV22 - Alunos - Vip esgotado</t>
+          <t>AD08 - Vídeo SAV22 - Pedro na arena</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -756,28 +756,28 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>2201.28</v>
+        <v>4802.21</v>
       </c>
       <c r="F7" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>41.53</v>
+        <v>85.75</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.02719343252950231</v>
+        <v>0.02873268342739867</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda LOTE 1 - FEV/24</t>
+          <t>[VENDAS] [AUTO] [Q] Venda LOTE 1 - FEV/24</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C3n5bofNQ9Z/</t>
+          <t>https://www.instagram.com/p/C3npkuBNMhG/</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -789,15 +789,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AD03 - Banner 3 Legenda 1</t>
+          <t>AD65 - Carrossel 4 - Palestrantes confirmados</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -806,28 +806,28 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>2879.85</v>
+        <v>934.12</v>
       </c>
       <c r="F8" t="n">
-        <v>145</v>
+        <v>53</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>19.86</v>
+        <v>17.62</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.06694367497691597</v>
+        <v>0.02719343252950231</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>[PRE-INSCRICOES] [CADASTROS] [AUTO] [Q] Pré-inscrições LOTE 1 - AGO/24</t>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] [V2] Venda LOTE 2 - MAI/24</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C-vBhFcMXZY/</t>
+          <t>https://www.instagram.com/p/C9c4mUht5FS/</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -839,45 +839,45 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AD03 - Banner 3 Legenda 4</t>
+          <t>AL01 - Vídeo SAV22 - Alunos - Vip esgotado</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>imagem</t>
+          <t>vídeo</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3102.87</v>
+        <v>2201.28</v>
       </c>
       <c r="F9" t="n">
-        <v>97</v>
+        <v>53</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>31.99</v>
+        <v>41.53</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.04478301015697138</v>
+        <v>0.02719343252950231</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda do LOTE 1 - ABR/25</t>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda LOTE 1 - FEV/24</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DJmClsQgfjL/</t>
+          <t>https://www.instagram.com/p/C3n5bofNQ9Z/</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -889,45 +889,45 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ADSUBIDO03 - Vídeo 9 Legenda 1 - Mexendo na amoeba</t>
+          <t>AD15 - Banner 8</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>vídeo</t>
+          <t>imagem</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>2628.39</v>
+        <v>2147.45</v>
       </c>
       <c r="F10" t="n">
-        <v>90</v>
+        <v>41</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>29.2</v>
+        <v>52.38</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.04155124653739612</v>
+        <v>0.02103642893791688</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda do LOTE 1 - ABR/25</t>
+          <t>[VENDAS] [AUTO] [Q] Venda LOTE 1 - FEV/24</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DJrWEvtsOJp/</t>
+          <t>https://www.instagram.com/p/C3sTI5mtfYR/</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -939,45 +939,45 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="B11" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>AD13 - Banner 6</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>2392.56</v>
+      </c>
+      <c r="F11" t="n">
+        <v>38</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>62.96</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>0.01949717804002052</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] Venda LOTE 1 - FEV/24</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
         <v>4</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>AD06 - Banner 3 Legenda 2</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>imagem</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>1674.12</v>
-      </c>
-      <c r="F11" t="n">
-        <v>73</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>22.93</v>
-      </c>
-      <c r="H11" s="3" t="n">
-        <v>0.03370267774699907</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>[PRE-INSCRICOES] [CADASTROS] [AUTO] [Q] Pré-inscrições LOTE 1 - AGO/24</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>3</v>
-      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C-vBgLpsp7v/</t>
+          <t>https://www.instagram.com/p/C3sTIpwtDrp/</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -989,37 +989,37 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AD29 - Vídeo 8 Legenda 4 - Sou o ingresso do SAV</t>
+          <t>AD16 - Banner 9</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>vídeo</t>
+          <t>imagem</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>2408.05</v>
+        <v>807.04</v>
       </c>
       <c r="F12" t="n">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>49.14</v>
+        <v>22.42</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.02262234533702678</v>
+        <v>0.01847101077475629</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda do LOTE 1 - ABR/25</t>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda LOTE 1 - FEV/24</t>
         </is>
       </c>
       <c r="J12" t="n">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DJrVZI3MB8V/</t>
+          <t>https://www.instagram.com/p/C56aBZItetJ/</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1039,7 +1039,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AD05_Banner_05_Ultimos_dias_Lote_1</t>
+          <t>AD03 - Banner 3 Legenda 1</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1056,20 +1056,20 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>3259.15</v>
+        <v>2879.85</v>
       </c>
       <c r="F13" t="n">
-        <v>100</v>
+        <v>145</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>32.59</v>
+        <v>19.86</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.06802721088435375</v>
+        <v>0.06694367497691597</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - JUN/26</t>
+          <t>[PRE-INSCRICOES] [CADASTROS] [AUTO] [Q] Pré-inscrições LOTE 1 - AGO/24</t>
         </is>
       </c>
       <c r="J13" t="n">
@@ -1077,19 +1077,19 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DZT4SE8DEV1/</t>
+          <t>https://www.instagram.com/p/C-vBhFcMXZY/</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>act_871468088416227</t>
+          <t>act_498598010251531</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1097,49 +1097,49 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AD13_Video_05_Sameday_Dia_1</t>
+          <t>AD03 - Banner 3 Legenda 4</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>vídeo</t>
+          <t>imagem</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>2012.14</v>
+        <v>3102.87</v>
       </c>
       <c r="F14" t="n">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>36.58</v>
+        <v>31.99</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.03741496598639456</v>
+        <v>0.04478301015697138</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - FEV/26</t>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda do LOTE 1 - ABR/25</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVJ00EYjGAz/</t>
+          <t>https://www.instagram.com/p/DJmClsQgfjL/</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>act_871468088416227</t>
+          <t>act_498598010251531</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1147,49 +1147,49 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AD10_Banner_07_Ultimos_dias_35_off</t>
+          <t>ADSUBIDO03 - Vídeo 9 Legenda 1 - Mexendo na amoeba</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>imagem</t>
+          <t>vídeo</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>1566.68</v>
+        <v>2628.39</v>
       </c>
       <c r="F15" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>39.17</v>
+        <v>29.2</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.0272108843537415</v>
+        <v>0.04155124653739612</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 4 - AGO/26</t>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda do LOTE 1 - ABR/25</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DbmkrdcsYdQ/</t>
+          <t>https://www.instagram.com/p/DJrWEvtsOJp/</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>act_871468088416227</t>
+          <t>act_498598010251531</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1197,29 +1197,29 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AD21_Video_09_Pedro_Ultimo_dia</t>
+          <t>AD22 - Banner 22 Legenda 4 - RJ continua subido V2</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>vídeo</t>
+          <t>imagem</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>1963.69</v>
+        <v>5794.69</v>
       </c>
       <c r="F16" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>49.09</v>
+        <v>77.26000000000001</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.0272108843537415</v>
+        <v>0.03462603878116344</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - AGO/25</t>
+          <t>[VENDAS] [AUTO] [Q] [REMARKETING] Venda do LOTE 1 - ABR/25</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -1227,19 +1227,19 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DN6ZK70jEDg/</t>
+          <t>https://www.instagram.com/p/DJRhJ6bs38k/</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>act_871468088416227</t>
+          <t>act_498598010251531</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1247,40 +1247,790 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>AD06 - Banner 3 Legenda 2</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>1674.12</v>
+      </c>
+      <c r="F17" t="n">
+        <v>73</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>22.93</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>0.03370267774699907</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>[PRE-INSCRICOES] [CADASTROS] [AUTO] [Q] Pré-inscrições LOTE 1 - AGO/24</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/C-vBgLpsp7v/</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>act_498598010251531</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>6</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>AD02 - Banner 2 Legenda 1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>4838.53</v>
+      </c>
+      <c r="F18" t="n">
+        <v>63</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>0.02908587257617729</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - AGO/24</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>6</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/C-zCYouMvNF/</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>act_498598010251531</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>7</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>AD29 - Vídeo 8 Legenda 4 - Sou o ingresso do SAV</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>vídeo</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>2408.05</v>
+      </c>
+      <c r="F19" t="n">
+        <v>49</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>49.14</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>0.02262234533702678</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda do LOTE 1 - ABR/25</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DJrVZI3MB8V/</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>act_498598010251531</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>AD10 - Banner 10 Legenda 2</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>2412.6</v>
+      </c>
+      <c r="F20" t="n">
+        <v>49</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>49.24</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>0.02262234533702678</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda do LOTE 1 - ABR/25</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>5</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DJZ_CNxgjv9/</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>act_498598010251531</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>9</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>AD10 - Banner 6 - Último dia Lote 1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>2437.78</v>
+      </c>
+      <c r="F21" t="n">
+        <v>45</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>54.17</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>0.02077562326869806</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - AGO/24</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>3</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/C--2XfPMycj/</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>act_498598010251531</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>10</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>AD08 - Banner 8 Legenda 3</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>2055.63</v>
+      </c>
+      <c r="F22" t="n">
+        <v>38</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>0.01754385964912281</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda do LOTE 1 - ABR/25</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>5</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DIgsH9IsUwZ/</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>act_498598010251531</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>AD05_Banner_05_Ultimos_dias_Lote_1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>3259.15</v>
+      </c>
+      <c r="F23" t="n">
+        <v>100</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>32.59</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>0.06802721088435375</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - JUN/26</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DZT4SE8DEV1/</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>act_871468088416227</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>AD13_Video_05_Sameday_Dia_1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>vídeo</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>2012.14</v>
+      </c>
+      <c r="F24" t="n">
+        <v>55</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>36.58</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>0.03741496598639456</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - FEV/26</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DVJ00EYjGAz/</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>act_871468088416227</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>AD10_Banner_07_Ultimos_dias_35_off</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>1566.68</v>
+      </c>
+      <c r="F25" t="n">
+        <v>40</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>39.17</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>0.0272108843537415</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 4 - AGO/26</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>3</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DbmkrdcsYdQ/</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>act_871468088416227</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>AD21_Video_09_Pedro_Ultimo_dia</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>vídeo</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>1963.69</v>
+      </c>
+      <c r="F26" t="n">
+        <v>40</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>49.09</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>0.0272108843537415</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - AGO/25</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>2</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DN6ZK70jEDg/</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>act_871468088416227</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>AD01_Banner_01_Lote_1_liberado</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>1887.03</v>
+      </c>
+      <c r="F27" t="n">
+        <v>34</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>0.02312925170068027</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - FEV/26</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>4</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DVJ1E8qDFOB/</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>act_871468088416227</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>AD01_Banner_01_Ultimos_dias_Lote_1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>2092.72</v>
+      </c>
+      <c r="F28" t="n">
+        <v>31</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>67.51000000000001</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>0.02108843537414966</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] [ALUNOS] Venda do LOTE 1 - JUN/26</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>2</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DZI0bQMjNqd/</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>act_871468088416227</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>7</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>AD04_Banner_04_Aberto_por_tempo_limitado</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>1818.63</v>
+      </c>
+      <c r="F29" t="n">
+        <v>30</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>60.62</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>0.02040816326530612</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - FEV/26</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>4</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DVJ1MFTDP5_/</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>act_871468088416227</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>8</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
           <t>AD20_Banner_09_Ultimo_dia_lote_1</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>imagem</t>
         </is>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E30" s="2" t="n">
         <v>859.13</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F30" t="n">
         <v>28</v>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="G30" s="2" t="n">
         <v>30.68</v>
       </c>
-      <c r="H17" s="3" t="n">
+      <c r="H30" s="3" t="n">
         <v>0.01904761904761905</v>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - AGO/25</t>
         </is>
       </c>
-      <c r="J17" t="n">
+      <c r="J30" t="n">
         <v>2</v>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>https://www.instagram.com/p/DN7FwNgDGMv/</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>act_871468088416227</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>9</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>AD19_Banner_08_Ultimo_dia_lote_1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>898.74</v>
+      </c>
+      <c r="F31" t="n">
+        <v>28</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>0.01904761904761905</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - AGO/25</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DN7FwZODK4g/</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>act_871468088416227</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>AD06_BN06_L03_SAV26_loves_SP</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>388.93</v>
+      </c>
+      <c r="F32" t="n">
+        <v>24</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>16.21</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>0.0163265306122449</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>[PRE-INSCRICOES] [CADASTROS] [AUTO] [Q] Remarketing - Pré-inscrições LOTE 1 - FEV/26</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>3</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DVGpukzjMIa/</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
         <is>
           <t>act_871468088416227</t>
         </is>
@@ -1408,11 +2158,11 @@
         <v>28</v>
       </c>
       <c r="G3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Sem concentração; mix natural do top 5. Top 1 = 15% das compras.</t>
+          <t>Sem concentração; mix natural do top 10. Top 1 = 15% das compras.</t>
         </is>
       </c>
     </row>
@@ -1438,11 +2188,11 @@
         <v>14</v>
       </c>
       <c r="G4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Sem concentração; mix natural do top 5. Top 1 = 7% das compras.</t>
+          <t>Sem concentração; mix natural do top 10. Top 1 = 7% das compras.</t>
         </is>
       </c>
     </row>
@@ -1468,11 +2218,11 @@
         <v>10</v>
       </c>
       <c r="G5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Sem concentração; mix natural do top 5. Top 1 = 7% das compras.</t>
+          <t>Sem concentração; mix natural do top 10. Top 1 = 7% das compras.</t>
         </is>
       </c>
     </row>
@@ -1524,7 +2274,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Concentração: se 1–3 anúncios somam &gt;=80% das compras do ano, lista só esses. Mix: se o top 5 é de um só tipo, entram os 2 melhores do outro tipo que atinjam o piso.</t>
+          <t>Concentração: se 1–3 anúncios somam &gt;=80% das compras do ano, lista só esses. Mix: se o top 10 é de um só tipo, entram os 3 melhores do outro tipo que atinjam o piso.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planilha por ano: apenas campanhas de VENDAS
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQAEiUYJHrFswFx8FRgado
</commit_message>
<xml_diff>
--- a/top_anuncios_subido_ao_vivo_por_ano.xlsx
+++ b/top_anuncios_subido_ao_vivo_por_ano.xlsx
@@ -556,16 +556,16 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>16570.55</v>
+        <v>14101.35</v>
       </c>
       <c r="F3" t="n">
         <v>285</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>58.14</v>
+        <v>49.48</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0.1462288353001539</v>
+        <v>0.1637931034482759</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -615,7 +615,7 @@
         <v>37.88</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.09338122113904566</v>
+        <v>0.1045977011494253</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -647,37 +647,37 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AD03 - Banner 2</t>
+          <t>AD08 - Vídeo SAV22 - Pedro na arena</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>imagem</t>
+          <t>vídeo</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>7060.98</v>
+        <v>4802.21</v>
       </c>
       <c r="F5" t="n">
-        <v>123</v>
+        <v>56</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>57.41</v>
+        <v>85.75</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.06310928681375064</v>
+        <v>0.03218390804597701</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>[PRE-INSCRICOES] [CADASTROS] [AUTO] [Q] Pré-inscrições LOTE 1 - FEV/24</t>
+          <t>[VENDAS] [AUTO] [Q] Venda LOTE 1 - FEV/24</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C3IGu_itq6v/</t>
+          <t>https://www.instagram.com/p/C3npkuBNMhG/</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -697,29 +697,29 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AD01 - Vídeo Feed 1</t>
+          <t>AD65 - Carrossel 4 - Palestrantes confirmados</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>vídeo</t>
+          <t>imagem</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>7980.04</v>
+        <v>934.12</v>
       </c>
       <c r="F6" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>137.59</v>
+        <v>17.62</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.0297588506926629</v>
+        <v>0.03045977011494253</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>[PRE-INSCRICOES] [CADASTROS] [AUTO] [Q] Pré-inscrições LOTE 1 - FEV/24</t>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] [V2] Venda LOTE 2 - MAI/24</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -727,7 +727,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C3FkNeQNkoM/</t>
+          <t>https://www.instagram.com/p/C9c4mUht5FS/</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AD08 - Vídeo SAV22 - Pedro na arena</t>
+          <t>AL01 - Vídeo SAV22 - Alunos - Vip esgotado</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -756,28 +756,28 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4802.21</v>
+        <v>2201.28</v>
       </c>
       <c r="F7" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>85.75</v>
+        <v>41.53</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.02873268342739867</v>
+        <v>0.03045977011494253</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] Venda LOTE 1 - FEV/24</t>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda LOTE 1 - FEV/24</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C3npkuBNMhG/</t>
+          <t>https://www.instagram.com/p/C3n5bofNQ9Z/</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AD65 - Carrossel 4 - Palestrantes confirmados</t>
+          <t>AD02 - Banner 2</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -806,28 +806,28 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>934.12</v>
+        <v>1885.66</v>
       </c>
       <c r="F8" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>17.62</v>
+        <v>40.12</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.02719343252950231</v>
+        <v>0.02701149425287356</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] [ALUNO] [V2] Venda LOTE 2 - MAI/24</t>
+          <t>[VENDAS] [AUTO] [Q] Venda LOTE 1 - FEV/24</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C9c4mUht5FS/</t>
+          <t>https://www.instagram.com/p/C3sTI5ON_p0/</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -847,37 +847,37 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AL01 - Vídeo SAV22 - Alunos - Vip esgotado</t>
+          <t>AD15 - Banner 8</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>vídeo</t>
+          <t>imagem</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>2201.28</v>
+        <v>2147.45</v>
       </c>
       <c r="F9" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>41.53</v>
+        <v>52.38</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.02719343252950231</v>
+        <v>0.0235632183908046</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda LOTE 1 - FEV/24</t>
+          <t>[VENDAS] [AUTO] [Q] Venda LOTE 1 - FEV/24</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C3n5bofNQ9Z/</t>
+          <t>https://www.instagram.com/p/C3sTI5mtfYR/</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AD15 - Banner 8</t>
+          <t>AD13 - Banner 6</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>2147.45</v>
+        <v>2392.56</v>
       </c>
       <c r="F10" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>52.38</v>
+        <v>62.96</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.02103642893791688</v>
+        <v>0.02183908045977011</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -923,11 +923,11 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C3sTI5mtfYR/</t>
+          <t>https://www.instagram.com/p/C3sTIpwtDrp/</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AD13 - Banner 6</t>
+          <t>AD16 - Banner 9</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -956,28 +956,28 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2392.56</v>
+        <v>807.04</v>
       </c>
       <c r="F11" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>62.96</v>
+        <v>22.42</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.01949717804002052</v>
+        <v>0.02068965517241379</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] Venda LOTE 1 - FEV/24</t>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda LOTE 1 - FEV/24</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C3sTIpwtDrp/</t>
+          <t>https://www.instagram.com/p/C56aBZItetJ/</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -997,25 +997,25 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AD16 - Banner 9</t>
+          <t>AL02 - Vídeo SAV22 - Alunos - Programação</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>imagem</t>
+          <t>vídeo</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>807.04</v>
+        <v>1014.93</v>
       </c>
       <c r="F12" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>22.42</v>
+        <v>36.25</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.01847101077475629</v>
+        <v>0.01609195402298851</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1023,11 +1023,11 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C56aBZItetJ/</t>
+          <t>https://www.instagram.com/p/C3n5bwQNfyX/</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AD03 - Banner 3 Legenda 1</t>
+          <t>AD03 - Banner 3 Legenda 4</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1056,28 +1056,28 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>2879.85</v>
+        <v>3102.87</v>
       </c>
       <c r="F13" t="n">
-        <v>145</v>
+        <v>97</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>19.86</v>
+        <v>31.99</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.06694367497691597</v>
+        <v>0.05452501405283867</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>[PRE-INSCRICOES] [CADASTROS] [AUTO] [Q] Pré-inscrições LOTE 1 - AGO/24</t>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda do LOTE 1 - ABR/25</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C-vBhFcMXZY/</t>
+          <t>https://www.instagram.com/p/DJmClsQgfjL/</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1097,25 +1097,25 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AD03 - Banner 3 Legenda 4</t>
+          <t>ADSUBIDO03 - Vídeo 9 Legenda 1 - Mexendo na amoeba</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>imagem</t>
+          <t>vídeo</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>3102.87</v>
+        <v>2628.39</v>
       </c>
       <c r="F14" t="n">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>31.99</v>
+        <v>29.2</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.04478301015697138</v>
+        <v>0.05059021922428331</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1123,11 +1123,11 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DJmClsQgfjL/</t>
+          <t>https://www.instagram.com/p/DJrWEvtsOJp/</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1147,37 +1147,37 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ADSUBIDO03 - Vídeo 9 Legenda 1 - Mexendo na amoeba</t>
+          <t>AD22 - Banner 22 Legenda 4 - RJ continua subido V2</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>vídeo</t>
+          <t>imagem</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>2628.39</v>
+        <v>5794.69</v>
       </c>
       <c r="F15" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>29.2</v>
+        <v>77.26000000000001</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.04155124653739612</v>
+        <v>0.04215851602023609</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda do LOTE 1 - ABR/25</t>
+          <t>[VENDAS] [AUTO] [Q] [REMARKETING] Venda do LOTE 1 - ABR/25</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DJrWEvtsOJp/</t>
+          <t>https://www.instagram.com/p/DJRhJ6bs38k/</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AD22 - Banner 22 Legenda 4 - RJ continua subido V2</t>
+          <t>AD02 - Banner 2 Legenda 1</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1206,28 +1206,28 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>5794.69</v>
+        <v>4311.14</v>
       </c>
       <c r="F16" t="n">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>77.26000000000001</v>
+        <v>74.33</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.03462603878116344</v>
+        <v>0.0326025857223159</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] [REMARKETING] Venda do LOTE 1 - ABR/25</t>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - AGO/24</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DJRhJ6bs38k/</t>
+          <t>https://www.instagram.com/p/C-zCYouMvNF/</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1247,37 +1247,37 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AD06 - Banner 3 Legenda 2</t>
+          <t>AD29 - Vídeo 8 Legenda 4 - Sou o ingresso do SAV</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>imagem</t>
+          <t>vídeo</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>1674.12</v>
+        <v>2408.05</v>
       </c>
       <c r="F17" t="n">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>22.93</v>
+        <v>49.14</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>0.03370267774699907</v>
+        <v>0.02754356379988758</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>[PRE-INSCRICOES] [CADASTROS] [AUTO] [Q] Pré-inscrições LOTE 1 - AGO/24</t>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda do LOTE 1 - ABR/25</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C-vBgLpsp7v/</t>
+          <t>https://www.instagram.com/p/DJrVZI3MB8V/</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AD02 - Banner 2 Legenda 1</t>
+          <t>AD10 - Banner 10 Legenda 2</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1306,28 +1306,28 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>4838.53</v>
+        <v>2412.6</v>
       </c>
       <c r="F18" t="n">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>76.8</v>
+        <v>49.24</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0.02908587257617729</v>
+        <v>0.02754356379988758</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - AGO/24</t>
+          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda do LOTE 1 - ABR/25</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C-zCYouMvNF/</t>
+          <t>https://www.instagram.com/p/DJZ_CNxgjv9/</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1347,37 +1347,37 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AD29 - Vídeo 8 Legenda 4 - Sou o ingresso do SAV</t>
+          <t>AD10 - Banner 6 - Último dia Lote 1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>vídeo</t>
+          <t>imagem</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>2408.05</v>
+        <v>2437.78</v>
       </c>
       <c r="F19" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>49.14</v>
+        <v>54.17</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>0.02262234533702678</v>
+        <v>0.02529510961214165</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] [ALUNO] Venda do LOTE 1 - ABR/25</t>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - AGO/24</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DJrVZI3MB8V/</t>
+          <t>https://www.instagram.com/p/C--2XfPMycj/</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AD10 - Banner 10 Legenda 2</t>
+          <t>AD08 - Banner 8 Legenda 3</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1406,16 +1406,16 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>2412.6</v>
+        <v>2055.63</v>
       </c>
       <c r="F20" t="n">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>49.24</v>
+        <v>54.1</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0.02262234533702678</v>
+        <v>0.02136031478358628</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DJZ_CNxgjv9/</t>
+          <t>https://www.instagram.com/p/DIgsH9IsUwZ/</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AD10 - Banner 6 - Último dia Lote 1</t>
+          <t>AD05 - Banner 5 Legenda 5</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1456,28 +1456,28 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>2437.78</v>
+        <v>1774.51</v>
       </c>
       <c r="F21" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>54.17</v>
+        <v>50.7</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.02077562326869806</v>
+        <v>0.01967397414277684</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - AGO/24</t>
+          <t>[VENDAS] [STORIES/REELS] [Q] Venda do LOTE 1 - FEV/25</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/C--2XfPMycj/</t>
+          <t>https://www.instagram.com/p/DGQ_Ov2sHrb/</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1497,25 +1497,25 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AD08 - Banner 8 Legenda 3</t>
+          <t>ADSUBIDO02 - Vídeo 1 Legenda 4 - Meu caro alunos da CST</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>imagem</t>
+          <t>vídeo</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>2055.63</v>
+        <v>1382.94</v>
       </c>
       <c r="F22" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>54.1</v>
+        <v>40.67</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0.01754385964912281</v>
+        <v>0.01911186059584036</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1523,11 +1523,11 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DIgsH9IsUwZ/</t>
+          <t>https://www.instagram.com/p/DJrVAK-sdOJ/</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -1565,7 +1565,7 @@
         <v>32.59</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0.06802721088435375</v>
+        <v>0.07867820613690008</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         <v>36.58</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>0.03741496598639456</v>
+        <v>0.04327301337529504</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1665,7 +1665,7 @@
         <v>39.17</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>0.0272108843537415</v>
+        <v>0.03147128245476003</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1715,7 +1715,7 @@
         <v>49.09</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0.0272108843537415</v>
+        <v>0.03147128245476003</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1765,7 +1765,7 @@
         <v>55.5</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>0.02312925170068027</v>
+        <v>0.02675059008654603</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AD01_Banner_01_Ultimos_dias_Lote_1</t>
+          <t>AD08_Banner_05_Black_esgotado</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1806,20 +1806,20 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>2092.72</v>
+        <v>2867.09</v>
       </c>
       <c r="F28" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>67.51000000000001</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>0.02108843537414966</v>
+        <v>0.02517702596380803</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] [ALUNOS] Venda do LOTE 1 - JUN/26</t>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - AGO/25</t>
         </is>
       </c>
       <c r="J28" t="n">
@@ -1827,7 +1827,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DZI0bQMjNqd/</t>
+          <t>https://www.instagram.com/p/DN3IIRx2PAQ/</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AD04_Banner_04_Aberto_por_tempo_limitado</t>
+          <t>AD01_Banner_01_Ultimos_dias_Lote_1</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1856,28 +1856,28 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>1818.63</v>
+        <v>2092.72</v>
       </c>
       <c r="F29" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>60.62</v>
+        <v>67.51000000000001</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.02040816326530612</v>
+        <v>0.02439024390243903</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - FEV/26</t>
+          <t>[VENDAS] [AUTO] [Q] [ALUNOS] Venda do LOTE 1 - JUN/26</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVJ1MFTDP5_/</t>
+          <t>https://www.instagram.com/p/DZI0bQMjNqd/</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AD20_Banner_09_Ultimo_dia_lote_1</t>
+          <t>AD04_Banner_04_Aberto_por_tempo_limitado</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1906,28 +1906,28 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>859.13</v>
+        <v>1818.63</v>
       </c>
       <c r="F30" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>30.68</v>
+        <v>60.62</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>0.01904761904761905</v>
+        <v>0.02360346184107003</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - AGO/25</t>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - FEV/26</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DN7FwNgDGMv/</t>
+          <t>https://www.instagram.com/p/DVJ1MFTDP5_/</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AD19_Banner_08_Ultimo_dia_lote_1</t>
+          <t>AD20_Banner_09_Ultimo_dia_lote_1</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1956,16 +1956,16 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>898.74</v>
+        <v>859.13</v>
       </c>
       <c r="F31" t="n">
         <v>28</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>32.1</v>
+        <v>30.68</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0.01904761904761905</v>
+        <v>0.02202989771833202</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DN7FwZODK4g/</t>
+          <t>https://www.instagram.com/p/DN7FwNgDGMv/</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AD06_BN06_L03_SAV26_loves_SP</t>
+          <t>AD19_Banner_08_Ultimo_dia_lote_1</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2006,28 +2006,28 @@
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>388.93</v>
+        <v>898.74</v>
       </c>
       <c r="F32" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>16.21</v>
+        <v>32.1</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>0.0163265306122449</v>
+        <v>0.02202989771833202</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>[PRE-INSCRICOES] [CADASTROS] [AUTO] [Q] Remarketing - Pré-inscrições LOTE 1 - FEV/26</t>
+          <t>[VENDAS] [AUTO] [Q] Venda do LOTE 1 - AGO/25</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DVGpukzjMIa/</t>
+          <t>https://www.instagram.com/p/DN7FwZODK4g/</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -2109,7 +2109,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>418.4</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Nenhuma compra registrada no ano (só campanhas de alcance/reconhecimento).</t>
+          <t>Sem campanhas de VENDAS no ano.</t>
         </is>
       </c>
     </row>
@@ -2143,13 +2143,13 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>147171.49</v>
+        <v>104751.41</v>
       </c>
       <c r="C3" t="n">
-        <v>1949</v>
+        <v>1740</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>75.51000000000001</v>
+        <v>60.2</v>
       </c>
       <c r="E3" t="n">
         <v>285</v>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Sem concentração; mix natural do top 10. Top 1 = 15% das compras.</t>
+          <t>Sem concentração; mix natural do top 10. Top 1 = 16% das compras.</t>
         </is>
       </c>
     </row>
@@ -2173,26 +2173,26 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>217819.41</v>
+        <v>178604.82</v>
       </c>
       <c r="C4" t="n">
-        <v>2166</v>
+        <v>1779</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>100.56</v>
+        <v>100.4</v>
       </c>
       <c r="E4" t="n">
-        <v>145</v>
+        <v>97</v>
       </c>
       <c r="F4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G4" t="n">
         <v>10</v>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Sem concentração; mix natural do top 10. Top 1 = 7% das compras.</t>
+          <t>Sem concentração; mix natural do top 10. Top 1 = 5% das compras.</t>
         </is>
       </c>
     </row>
@@ -2203,13 +2203,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>145239.99</v>
+        <v>115908.1</v>
       </c>
       <c r="C5" t="n">
-        <v>1470</v>
+        <v>1271</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>98.8</v>
+        <v>91.19</v>
       </c>
       <c r="E5" t="n">
         <v>100</v>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Sem concentração; mix natural do top 10. Top 1 = 7% das compras.</t>
+          <t>Sem concentração; mix natural do top 10. Top 1 = 8% das compras.</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2246,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Fonte: extração do Stract (campanhas '[SUBIDO AO VIVO AAAA]', contas act_498598010251531 e act_871468088416227). Ano = o que está entre colchetes no nome da campanha (ex.: campanha '[SUBIDO AO VIVO 2025] ... LOTE 1 - AGO/24' conta como 2025).</t>
+          <t>Filtro: apenas campanhas com [VENDAS] no nome (pré-inscrições, alcance, engajamento, tráfego, aquecimento etc. excluídas). Fonte: extração do Stract (campanhas '[SUBIDO AO VIVO AAAA]', contas act_498598010251531 e act_871468088416227). Ano = o que está entre colchetes no nome da campanha (ex.: campanha '[SUBIDO AO VIVO 2025] ... LOTE 1 - AGO/24' conta como 2025).</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2295,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2023: só há campanha de reconhecimento (carrossel) sem compras. 2026: dados até 02/10/2026.</t>
+          <t>2023: não há campanha de vendas na extração. 2026: dados até 02/10/2026.</t>
         </is>
       </c>
     </row>

</xml_diff>